<commit_message>
GamePageDTO allUser attribute typo
</commit_message>
<xml_diff>
--- a/SquashPlanner.xlsx
+++ b/SquashPlanner.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Programozas\Java_Oktatas\Java_Halado\Nagyfeladatok\Squash\Repo\jft8_squash\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7F0E0A87-568E-49E3-AB47-81DFEC32FA42}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F75158AD-3A4E-461A-B0AB-35C3A2BEAED0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="16440" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="16440" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="DB" sheetId="1" r:id="rId1"/>
@@ -278,11 +278,6 @@
     <t>GamePageDTO</t>
   </si>
   <si>
-    <t>games::List&lt;GameDTO&gt;
-allUuser::List&lt;UserDTO&gt;
-allPlace::List&lt;PlaceDTO&gt;</t>
-  </si>
-  <si>
     <t>id::Int
 name::String</t>
   </si>
@@ -411,16 +406,29 @@
   <si>
     <t>AdminService</t>
   </si>
+  <si>
+    <t>games::List&lt;GameDTO&gt;
+allUser::List&lt;UserDTO&gt;
+allPlace::List&lt;PlaceDTO&gt;</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="13" x14ac:knownFonts="1">
+  <fonts count="14" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="238"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -574,81 +582,69 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="34">
+  <cellXfs count="35">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -657,14 +653,29 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normál" xfId="0" builtinId="0"/>
@@ -895,10 +906,10 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="17" t="s">
+      <c r="A1" s="30" t="s">
         <v>11</v>
       </c>
-      <c r="B1" s="18" t="s">
+      <c r="B1" s="31" t="s">
         <v>12</v>
       </c>
       <c r="C1" s="16" t="s">
@@ -912,8 +923,8 @@
       </c>
     </row>
     <row r="2" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="17"/>
-      <c r="B2" s="18"/>
+      <c r="A2" s="30"/>
+      <c r="B2" s="31"/>
       <c r="C2" s="15" t="s">
         <v>13</v>
       </c>
@@ -922,8 +933,8 @@
       </c>
     </row>
     <row r="3" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="17"/>
-      <c r="B3" s="18"/>
+      <c r="A3" s="30"/>
+      <c r="B3" s="31"/>
       <c r="C3" s="15" t="s">
         <v>14</v>
       </c>
@@ -932,8 +943,8 @@
       </c>
     </row>
     <row r="4" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="17"/>
-      <c r="B4" s="18"/>
+      <c r="A4" s="30"/>
+      <c r="B4" s="31"/>
       <c r="C4" s="15" t="s">
         <v>15</v>
       </c>
@@ -942,8 +953,8 @@
       </c>
     </row>
     <row r="5" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="17"/>
-      <c r="B5" s="18"/>
+      <c r="A5" s="30"/>
+      <c r="B5" s="31"/>
       <c r="C5" s="15" t="s">
         <v>16</v>
       </c>
@@ -952,8 +963,8 @@
       </c>
     </row>
     <row r="6" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="17"/>
-      <c r="B6" s="18"/>
+      <c r="A6" s="30"/>
+      <c r="B6" s="31"/>
       <c r="C6" s="15" t="s">
         <v>34</v>
       </c>
@@ -965,8 +976,8 @@
       </c>
     </row>
     <row r="7" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="17"/>
-      <c r="B7" s="18" t="s">
+      <c r="A7" s="30"/>
+      <c r="B7" s="31" t="s">
         <v>22</v>
       </c>
       <c r="C7" s="16" t="s">
@@ -980,8 +991,8 @@
       </c>
     </row>
     <row r="8" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="17"/>
-      <c r="B8" s="18"/>
+      <c r="A8" s="30"/>
+      <c r="B8" s="31"/>
       <c r="C8" s="15" t="s">
         <v>13</v>
       </c>
@@ -990,8 +1001,8 @@
       </c>
     </row>
     <row r="9" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="17"/>
-      <c r="B9" s="18"/>
+      <c r="A9" s="30"/>
+      <c r="B9" s="31"/>
       <c r="C9" s="15" t="s">
         <v>23</v>
       </c>
@@ -1000,8 +1011,8 @@
       </c>
     </row>
     <row r="10" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="17"/>
-      <c r="B10" s="18"/>
+      <c r="A10" s="30"/>
+      <c r="B10" s="31"/>
       <c r="C10" s="15" t="s">
         <v>24</v>
       </c>
@@ -1010,8 +1021,8 @@
       </c>
     </row>
     <row r="11" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="17"/>
-      <c r="B11" s="18" t="s">
+      <c r="A11" s="30"/>
+      <c r="B11" s="31" t="s">
         <v>25</v>
       </c>
       <c r="C11" s="16" t="s">
@@ -1025,8 +1036,8 @@
       </c>
     </row>
     <row r="12" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="17"/>
-      <c r="B12" s="18"/>
+      <c r="A12" s="30"/>
+      <c r="B12" s="31"/>
       <c r="C12" s="15" t="s">
         <v>26</v>
       </c>
@@ -1038,8 +1049,8 @@
       </c>
     </row>
     <row r="13" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="17"/>
-      <c r="B13" s="18"/>
+      <c r="A13" s="30"/>
+      <c r="B13" s="31"/>
       <c r="C13" s="15" t="s">
         <v>27</v>
       </c>
@@ -1051,8 +1062,8 @@
       </c>
     </row>
     <row r="14" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="17"/>
-      <c r="B14" s="18"/>
+      <c r="A14" s="30"/>
+      <c r="B14" s="31"/>
       <c r="C14" s="15" t="s">
         <v>28</v>
       </c>
@@ -1061,8 +1072,8 @@
       </c>
     </row>
     <row r="15" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="17"/>
-      <c r="B15" s="18"/>
+      <c r="A15" s="30"/>
+      <c r="B15" s="31"/>
       <c r="C15" s="15" t="s">
         <v>29</v>
       </c>
@@ -1071,8 +1082,8 @@
       </c>
     </row>
     <row r="16" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="17"/>
-      <c r="B16" s="18"/>
+      <c r="A16" s="30"/>
+      <c r="B16" s="31"/>
       <c r="C16" s="15" t="s">
         <v>30</v>
       </c>
@@ -1084,8 +1095,8 @@
       </c>
     </row>
     <row r="17" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="17"/>
-      <c r="B17" s="18"/>
+      <c r="A17" s="30"/>
+      <c r="B17" s="31"/>
       <c r="C17" s="15" t="s">
         <v>32</v>
       </c>
@@ -2039,7 +2050,7 @@
   <cols>
     <col min="1" max="2" width="20.88671875" customWidth="1"/>
     <col min="3" max="3" width="15.88671875" customWidth="1"/>
-    <col min="4" max="4" width="25.88671875" style="29" customWidth="1"/>
+    <col min="4" max="4" width="25.88671875" style="25" customWidth="1"/>
     <col min="5" max="5" width="45.77734375" customWidth="1"/>
     <col min="6" max="6" width="26.88671875" customWidth="1"/>
     <col min="7" max="7" width="28.88671875" customWidth="1"/>
@@ -2057,7 +2068,7 @@
       <c r="C1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="25" t="s">
+      <c r="D1" s="21" t="s">
         <v>2</v>
       </c>
       <c r="E1" s="1" t="s">
@@ -2069,7 +2080,7 @@
       <c r="G1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="H1" s="31" t="s">
+      <c r="H1" s="27" t="s">
         <v>6</v>
       </c>
     </row>
@@ -2083,7 +2094,7 @@
       <c r="C2" s="11" t="s">
         <v>38</v>
       </c>
-      <c r="D2" s="26" t="s">
+      <c r="D2" s="22" t="s">
         <v>39</v>
       </c>
       <c r="E2" s="11" t="s">
@@ -2095,160 +2106,160 @@
       <c r="G2" s="11" t="s">
         <v>36</v>
       </c>
-      <c r="H2" s="24" t="s">
-        <v>91</v>
+      <c r="H2" s="20" t="s">
+        <v>90</v>
       </c>
     </row>
     <row r="3" spans="1:8" s="4" customFormat="1" ht="44.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="21" t="s">
+      <c r="A3" s="32" t="s">
         <v>40</v>
       </c>
-      <c r="B3" s="21" t="s">
+      <c r="B3" s="32" t="s">
         <v>41</v>
       </c>
-      <c r="C3" s="21" t="s">
+      <c r="C3" s="32" t="s">
         <v>42</v>
       </c>
-      <c r="D3" s="22" t="s">
+      <c r="D3" s="33" t="s">
         <v>43</v>
       </c>
-      <c r="E3" s="22" t="s">
+      <c r="E3" s="33" t="s">
         <v>44</v>
       </c>
-      <c r="F3" s="20" t="s">
+      <c r="F3" s="18" t="s">
         <v>46</v>
       </c>
-      <c r="G3" s="20" t="s">
+      <c r="G3" s="18" t="s">
         <v>58</v>
       </c>
-      <c r="H3" s="32" t="s">
+      <c r="H3" s="28" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" s="4" customFormat="1" ht="46.2" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="32"/>
+      <c r="B4" s="32"/>
+      <c r="C4" s="32"/>
+      <c r="D4" s="33"/>
+      <c r="E4" s="33"/>
+      <c r="F4" s="18" t="s">
+        <v>45</v>
+      </c>
+      <c r="G4" s="17" t="s">
+        <v>50</v>
+      </c>
+      <c r="H4" s="28" t="s">
         <v>87</v>
       </c>
     </row>
-    <row r="4" spans="1:8" s="4" customFormat="1" ht="46.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="21"/>
-      <c r="B4" s="21"/>
-      <c r="C4" s="21"/>
-      <c r="D4" s="22"/>
-      <c r="E4" s="22"/>
-      <c r="F4" s="20" t="s">
-        <v>45</v>
-      </c>
-      <c r="G4" s="19" t="s">
+    <row r="5" spans="1:8" s="4" customFormat="1" ht="38.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="32"/>
+      <c r="B5" s="32"/>
+      <c r="C5" s="32"/>
+      <c r="D5" s="33"/>
+      <c r="E5" s="33"/>
+      <c r="F5" s="18" t="s">
+        <v>47</v>
+      </c>
+      <c r="G5" s="17" t="s">
         <v>50</v>
       </c>
-      <c r="H4" s="32" t="s">
+      <c r="H5" s="28" t="s">
         <v>88</v>
       </c>
     </row>
-    <row r="5" spans="1:8" s="4" customFormat="1" ht="38.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="21"/>
-      <c r="B5" s="21"/>
-      <c r="C5" s="21"/>
-      <c r="D5" s="22"/>
-      <c r="E5" s="22"/>
-      <c r="F5" s="20" t="s">
-        <v>47</v>
-      </c>
-      <c r="G5" s="19" t="s">
-        <v>50</v>
-      </c>
-      <c r="H5" s="32" t="s">
+    <row r="6" spans="1:8" s="4" customFormat="1" ht="44.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="32"/>
+      <c r="B6" s="32"/>
+      <c r="C6" s="32"/>
+      <c r="D6" s="33"/>
+      <c r="E6" s="33"/>
+      <c r="F6" s="18" t="s">
+        <v>48</v>
+      </c>
+      <c r="G6" s="17" t="s">
+        <v>52</v>
+      </c>
+      <c r="H6" s="28" t="s">
         <v>89</v>
       </c>
     </row>
-    <row r="6" spans="1:8" s="4" customFormat="1" ht="44.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="21"/>
-      <c r="B6" s="21"/>
-      <c r="C6" s="21"/>
-      <c r="D6" s="22"/>
-      <c r="E6" s="22"/>
-      <c r="F6" s="20" t="s">
-        <v>48</v>
-      </c>
-      <c r="G6" s="19" t="s">
-        <v>52</v>
-      </c>
-      <c r="H6" s="32" t="s">
+    <row r="7" spans="1:8" s="4" customFormat="1" ht="44.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="17" t="s">
+        <v>61</v>
+      </c>
+      <c r="B7" s="17" t="s">
+        <v>76</v>
+      </c>
+      <c r="C7" s="17" t="s">
+        <v>42</v>
+      </c>
+      <c r="D7" s="18" t="s">
+        <v>62</v>
+      </c>
+      <c r="E7" s="18" t="s">
+        <v>63</v>
+      </c>
+      <c r="F7" s="17" t="s">
+        <v>64</v>
+      </c>
+      <c r="G7" s="18" t="s">
+        <v>58</v>
+      </c>
+      <c r="H7" s="28" t="s">
         <v>90</v>
       </c>
     </row>
-    <row r="7" spans="1:8" s="4" customFormat="1" ht="44.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="19" t="s">
-        <v>62</v>
-      </c>
-      <c r="B7" s="19" t="s">
+    <row r="8" spans="1:8" s="4" customFormat="1" ht="51.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="17" t="s">
+        <v>64</v>
+      </c>
+      <c r="B8" s="17" t="s">
         <v>77</v>
       </c>
-      <c r="C7" s="19" t="s">
-        <v>42</v>
-      </c>
-      <c r="D7" s="20" t="s">
-        <v>63</v>
-      </c>
-      <c r="E7" s="20" t="s">
+      <c r="C8" s="17" t="s">
+        <v>38</v>
+      </c>
+      <c r="D8" s="18" t="s">
+        <v>65</v>
+      </c>
+      <c r="E8" s="18" t="s">
+        <v>67</v>
+      </c>
+      <c r="F8" s="17" t="s">
         <v>64</v>
       </c>
-      <c r="F7" s="19" t="s">
-        <v>65</v>
-      </c>
-      <c r="G7" s="20" t="s">
+      <c r="G8" s="18" t="s">
         <v>58</v>
       </c>
-      <c r="H7" s="32" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="8" spans="1:8" s="4" customFormat="1" ht="51.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="19" t="s">
-        <v>65</v>
-      </c>
-      <c r="B8" s="19" t="s">
+      <c r="H8" s="28" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" s="4" customFormat="1" ht="51.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A9" s="17" t="s">
+        <v>64</v>
+      </c>
+      <c r="B9" s="17" t="s">
         <v>78</v>
       </c>
-      <c r="C8" s="19" t="s">
+      <c r="C9" s="17" t="s">
         <v>38</v>
       </c>
-      <c r="D8" s="20" t="s">
+      <c r="D9" s="18" t="s">
         <v>66</v>
       </c>
-      <c r="E8" s="20" t="s">
+      <c r="E9" s="18" t="s">
         <v>68</v>
       </c>
-      <c r="F8" s="19" t="s">
-        <v>65</v>
-      </c>
-      <c r="G8" s="20" t="s">
+      <c r="F9" s="17" t="s">
+        <v>64</v>
+      </c>
+      <c r="G9" s="18" t="s">
         <v>58</v>
       </c>
-      <c r="H8" s="32" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="9" spans="1:8" s="4" customFormat="1" ht="51.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A9" s="19" t="s">
-        <v>65</v>
-      </c>
-      <c r="B9" s="19" t="s">
-        <v>79</v>
-      </c>
-      <c r="C9" s="19" t="s">
-        <v>38</v>
-      </c>
-      <c r="D9" s="20" t="s">
-        <v>67</v>
-      </c>
-      <c r="E9" s="20" t="s">
-        <v>69</v>
-      </c>
-      <c r="F9" s="19" t="s">
-        <v>65</v>
-      </c>
-      <c r="G9" s="20" t="s">
-        <v>58</v>
-      </c>
-      <c r="H9" s="32" t="s">
-        <v>87</v>
+      <c r="H9" s="28" t="s">
+        <v>86</v>
       </c>
     </row>
     <row r="10" spans="1:8" s="4" customFormat="1" ht="63" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
@@ -2264,94 +2275,94 @@
       <c r="A11" s="3"/>
       <c r="B11" s="3"/>
       <c r="C11" s="3"/>
-      <c r="D11" s="27"/>
+      <c r="D11" s="23"/>
       <c r="E11" s="3"/>
       <c r="F11" s="3"/>
       <c r="G11" s="3"/>
     </row>
     <row r="12" spans="1:8" ht="49.2" customHeight="1" thickTop="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="30" t="s">
+      <c r="A12" s="26" t="s">
+        <v>69</v>
+      </c>
+      <c r="B12" s="5" t="s">
+        <v>73</v>
+      </c>
+      <c r="C12" s="26" t="s">
+        <v>42</v>
+      </c>
+      <c r="D12" s="19" t="s">
         <v>70</v>
       </c>
-      <c r="B12" s="5" t="s">
+      <c r="E12" s="19" t="s">
+        <v>79</v>
+      </c>
+      <c r="F12" s="26" t="s">
+        <v>69</v>
+      </c>
+      <c r="G12" s="17" t="s">
+        <v>50</v>
+      </c>
+      <c r="H12" s="28" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" ht="39.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A13" s="17" t="s">
+        <v>69</v>
+      </c>
+      <c r="B13" s="17" t="s">
         <v>74</v>
       </c>
-      <c r="C12" s="30" t="s">
+      <c r="C13" s="17" t="s">
         <v>42</v>
       </c>
-      <c r="D12" s="23" t="s">
+      <c r="D13" s="18" t="s">
         <v>71</v>
       </c>
-      <c r="E12" s="23" t="s">
+      <c r="E13" s="18" t="s">
+        <v>84</v>
+      </c>
+      <c r="F13" s="26" t="s">
+        <v>69</v>
+      </c>
+      <c r="G13" s="17" t="s">
+        <v>50</v>
+      </c>
+      <c r="H13" s="28" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" ht="39" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A14" s="26" t="s">
+        <v>69</v>
+      </c>
+      <c r="B14" s="5" t="s">
+        <v>75</v>
+      </c>
+      <c r="C14" s="26" t="s">
+        <v>42</v>
+      </c>
+      <c r="D14" s="19" t="s">
+        <v>72</v>
+      </c>
+      <c r="E14" s="19" t="s">
         <v>80</v>
       </c>
-      <c r="F12" s="30" t="s">
-        <v>70</v>
-      </c>
-      <c r="G12" s="19" t="s">
+      <c r="F14" s="26" t="s">
+        <v>69</v>
+      </c>
+      <c r="G14" s="17" t="s">
         <v>50</v>
       </c>
-      <c r="H12" s="32" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="13" spans="1:8" ht="39.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="19" t="s">
-        <v>70</v>
-      </c>
-      <c r="B13" s="19" t="s">
-        <v>75</v>
-      </c>
-      <c r="C13" s="19" t="s">
-        <v>42</v>
-      </c>
-      <c r="D13" s="20" t="s">
-        <v>72</v>
-      </c>
-      <c r="E13" s="20" t="s">
-        <v>85</v>
-      </c>
-      <c r="F13" s="30" t="s">
-        <v>70</v>
-      </c>
-      <c r="G13" s="19" t="s">
-        <v>50</v>
-      </c>
-      <c r="H13" s="32" t="s">
+      <c r="H14" s="28" t="s">
         <v>88</v>
-      </c>
-    </row>
-    <row r="14" spans="1:8" ht="39" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A14" s="30" t="s">
-        <v>70</v>
-      </c>
-      <c r="B14" s="5" t="s">
-        <v>76</v>
-      </c>
-      <c r="C14" s="30" t="s">
-        <v>42</v>
-      </c>
-      <c r="D14" s="23" t="s">
-        <v>73</v>
-      </c>
-      <c r="E14" s="23" t="s">
-        <v>81</v>
-      </c>
-      <c r="F14" s="30" t="s">
-        <v>70</v>
-      </c>
-      <c r="G14" s="19" t="s">
-        <v>50</v>
-      </c>
-      <c r="H14" s="32" t="s">
-        <v>89</v>
       </c>
     </row>
     <row r="15" spans="1:8" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A15" s="3"/>
       <c r="B15" s="3"/>
       <c r="C15" s="3"/>
-      <c r="D15" s="27"/>
+      <c r="D15" s="23"/>
       <c r="E15" s="3"/>
       <c r="F15" s="3"/>
       <c r="G15" s="3"/>
@@ -2360,25 +2371,25 @@
       <c r="A16" s="10"/>
       <c r="B16" s="2"/>
       <c r="C16" s="10"/>
-      <c r="D16" s="28"/>
-      <c r="E16" s="30" t="s">
-        <v>86</v>
-      </c>
-      <c r="F16" s="30" t="s">
+      <c r="D16" s="24"/>
+      <c r="E16" s="26" t="s">
+        <v>85</v>
+      </c>
+      <c r="F16" s="26" t="s">
         <v>40</v>
       </c>
-      <c r="G16" s="30" t="s">
+      <c r="G16" s="26" t="s">
         <v>50</v>
       </c>
-      <c r="H16" s="32" t="s">
-        <v>90</v>
+      <c r="H16" s="28" t="s">
+        <v>89</v>
       </c>
     </row>
     <row r="17" spans="1:7" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A17" s="10"/>
       <c r="B17" s="2"/>
       <c r="C17" s="10"/>
-      <c r="D17" s="28"/>
+      <c r="D17" s="24"/>
       <c r="E17" s="10"/>
       <c r="F17" s="10"/>
       <c r="G17" s="10"/>
@@ -2387,7 +2398,7 @@
       <c r="A18" s="10"/>
       <c r="B18" s="2"/>
       <c r="C18" s="10"/>
-      <c r="D18" s="28"/>
+      <c r="D18" s="24"/>
       <c r="E18" s="10"/>
       <c r="F18" s="10"/>
       <c r="G18" s="10"/>
@@ -2396,7 +2407,7 @@
       <c r="A19" s="10"/>
       <c r="B19" s="2"/>
       <c r="C19" s="10"/>
-      <c r="D19" s="28"/>
+      <c r="D19" s="24"/>
       <c r="E19" s="10"/>
       <c r="F19" s="10"/>
       <c r="G19" s="10"/>
@@ -2405,7 +2416,7 @@
       <c r="A20" s="10"/>
       <c r="B20" s="2"/>
       <c r="C20" s="10"/>
-      <c r="D20" s="28"/>
+      <c r="D20" s="24"/>
       <c r="E20" s="10"/>
       <c r="F20" s="10"/>
       <c r="G20" s="10"/>
@@ -2414,7 +2425,7 @@
       <c r="A21" s="10"/>
       <c r="B21" s="2"/>
       <c r="C21" s="10"/>
-      <c r="D21" s="28"/>
+      <c r="D21" s="24"/>
       <c r="E21" s="10"/>
       <c r="F21" s="10"/>
       <c r="G21" s="10"/>
@@ -5385,88 +5396,88 @@
       <c r="A2" s="7" t="s">
         <v>50</v>
       </c>
-      <c r="B2" s="23" t="s">
+      <c r="B2" s="19" t="s">
         <v>51</v>
       </c>
-      <c r="C2" s="32" t="s">
-        <v>87</v>
+      <c r="C2" s="28" t="s">
+        <v>86</v>
       </c>
     </row>
     <row r="3" spans="1:3" ht="72.599999999999994" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="7" t="s">
         <v>58</v>
       </c>
-      <c r="B3" s="23" t="s">
-        <v>59</v>
-      </c>
-      <c r="C3" s="32" t="s">
-        <v>88</v>
+      <c r="B3" s="34" t="s">
+        <v>97</v>
+      </c>
+      <c r="C3" s="28" t="s">
+        <v>87</v>
       </c>
     </row>
     <row r="4" spans="1:3" ht="96" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="7" t="s">
         <v>49</v>
       </c>
-      <c r="B4" s="23" t="s">
+      <c r="B4" s="19" t="s">
         <v>57</v>
       </c>
-      <c r="C4" s="32" t="s">
-        <v>91</v>
+      <c r="C4" s="28" t="s">
+        <v>90</v>
       </c>
     </row>
     <row r="5" spans="1:3" ht="35.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="7" t="s">
         <v>52</v>
       </c>
-      <c r="B5" s="23" t="s">
-        <v>60</v>
-      </c>
-      <c r="C5" s="32" t="s">
-        <v>90</v>
+      <c r="B5" s="19" t="s">
+        <v>59</v>
+      </c>
+      <c r="C5" s="28" t="s">
+        <v>89</v>
       </c>
     </row>
     <row r="6" spans="1:3" ht="51.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="7" t="s">
         <v>53</v>
       </c>
-      <c r="B6" s="23" t="s">
+      <c r="B6" s="19" t="s">
         <v>54</v>
       </c>
-      <c r="C6" s="32" t="s">
-        <v>89</v>
+      <c r="C6" s="28" t="s">
+        <v>88</v>
       </c>
     </row>
     <row r="7" spans="1:3" ht="75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="7" t="s">
         <v>55</v>
       </c>
-      <c r="B7" s="23" t="s">
-        <v>61</v>
-      </c>
-      <c r="C7" s="32" t="s">
-        <v>87</v>
+      <c r="B7" s="19" t="s">
+        <v>60</v>
+      </c>
+      <c r="C7" s="28" t="s">
+        <v>86</v>
       </c>
     </row>
     <row r="8" spans="1:3" ht="103.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="7" t="s">
-        <v>83</v>
-      </c>
-      <c r="B8" s="23" t="s">
         <v>82</v>
       </c>
-      <c r="C8" s="32" t="s">
-        <v>88</v>
+      <c r="B8" s="19" t="s">
+        <v>81</v>
+      </c>
+      <c r="C8" s="28" t="s">
+        <v>87</v>
       </c>
     </row>
     <row r="9" spans="1:3" ht="52.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="7" t="s">
-        <v>84</v>
-      </c>
-      <c r="B9" s="23" t="s">
+        <v>83</v>
+      </c>
+      <c r="B9" s="19" t="s">
         <v>56</v>
       </c>
-      <c r="C9" s="32" t="s">
-        <v>91</v>
+      <c r="C9" s="28" t="s">
+        <v>90</v>
       </c>
     </row>
   </sheetData>
@@ -5494,51 +5505,51 @@
       </c>
     </row>
     <row r="2" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="33" t="s">
+      <c r="A2" s="29" t="s">
+        <v>93</v>
+      </c>
+      <c r="B2" s="29" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="29" t="s">
         <v>94</v>
       </c>
-      <c r="B2" s="33" t="s">
+      <c r="B3" s="29" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="29" t="s">
+        <v>95</v>
+      </c>
+      <c r="B4" s="29" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="29" t="s">
+        <v>96</v>
+      </c>
+      <c r="B5" s="29" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A6" s="29" t="s">
         <v>91</v>
       </c>
-    </row>
-    <row r="3" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="33" t="s">
-        <v>95</v>
-      </c>
-      <c r="B3" s="33" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="33" t="s">
-        <v>96</v>
-      </c>
-      <c r="B4" s="33" t="s">
+      <c r="B6" s="29" t="s">
         <v>87</v>
       </c>
     </row>
-    <row r="5" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="33" t="s">
-        <v>97</v>
-      </c>
-      <c r="B5" s="33" t="s">
+    <row r="7" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="28" t="s">
+        <v>92</v>
+      </c>
+      <c r="B7" s="28" t="s">
         <v>90</v>
-      </c>
-    </row>
-    <row r="6" spans="1:2" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A6" s="33" t="s">
-        <v>92</v>
-      </c>
-      <c r="B6" s="33" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="7" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="32" t="s">
-        <v>93</v>
-      </c>
-      <c r="B7" s="32" t="s">
-        <v>91</v>
       </c>
     </row>
     <row r="8" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.3">

</xml_diff>